<commit_message>
good progress on updated restart broken
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/restart_broken/NEW_PARAMS.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/restart_broken/NEW_PARAMS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\restart_broken\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B15585C-5598-4025-95E9-085D6F82A2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06AF9BAA-707A-4D8E-8956-4BCAF1AEC016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="44">
   <si>
     <t>-------------------</t>
   </si>
@@ -166,27 +166,6 @@
   </si>
   <si>
     <t>for 45° slope</t>
-  </si>
-  <si>
-    <t>NEW_PARAMS</t>
-  </si>
-  <si>
-    <t>classic_spinup</t>
-  </si>
-  <si>
-    <t>num_loops</t>
-  </si>
-  <si>
-    <t>1 if user wants a classic spinup</t>
-  </si>
-  <si>
-    <t>number of iterations of the classic spinup</t>
-  </si>
-  <si>
-    <t>accelerated_spinup</t>
-  </si>
-  <si>
-    <t>1 if user wants an accelerated spinup</t>
   </si>
 </sst>
 </file>
@@ -240,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -258,7 +237,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.54296875" style="1" customWidth="1"/>
@@ -591,435 +569,380 @@
     <col min="13" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2840</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="5"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="5"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D13" s="5"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D14" s="5"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="1">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35"/>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1958</v>
+      </c>
+      <c r="D27" s="1">
+        <v>8</v>
+      </c>
+      <c r="E27" s="1">
+        <v>29</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="1">
+        <v>1959</v>
+      </c>
+      <c r="D28" s="1">
+        <v>9</v>
+      </c>
+      <c r="E28" s="1">
+        <v>2</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="1">
+      <c r="B34" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B37" s="1">
         <v>0</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="C37" s="1">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B38" s="1">
+        <v>100</v>
+      </c>
+      <c r="C38" s="1">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B39" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" outlineLevel="1" x14ac:dyDescent="0.35"/>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+    <row r="43" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="1">
-        <v>45.3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="1">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="1">
-        <v>2840</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="3">
+    <row r="44" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>31</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>32</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="D45" s="6"/>
+    </row>
+    <row r="46" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>33</v>
+      </c>
+      <c r="B46">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="5"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+      <c r="D46" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H46" s="6"/>
+    </row>
+    <row r="47" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47">
+        <v>2844</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48">
+        <v>2790</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>2</v>
       </c>
-      <c r="D21" s="5"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D22" s="5"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="D23" s="5"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B26" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="1">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
+    </row>
+    <row r="50" spans="1:4" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:4" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="52" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D52" s="6"/>
+    </row>
+    <row r="53" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1</v>
+      </c>
+      <c r="D53" s="6"/>
+    </row>
+    <row r="54" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>41</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="D54" s="6"/>
+    </row>
+    <row r="55" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B55" s="7">
+        <v>3034</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35"/>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C36" s="1">
-        <v>1958</v>
-      </c>
-      <c r="D36" s="1">
-        <v>8</v>
-      </c>
-      <c r="E36" s="1">
-        <v>29</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C37" s="1">
-        <v>1959</v>
-      </c>
-      <c r="D37" s="1">
-        <v>9</v>
-      </c>
-      <c r="E37" s="1">
-        <v>2</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B43" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B46" s="1">
-        <v>0</v>
-      </c>
-      <c r="C46" s="1">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B47" s="1">
-        <v>100</v>
-      </c>
-      <c r="C47" s="1">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B48" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>31</v>
-      </c>
-      <c r="B53" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>32</v>
-      </c>
-      <c r="B54">
-        <v>1</v>
-      </c>
-      <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>33</v>
-      </c>
-      <c r="B55">
-        <v>0</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H55" s="6"/>
-    </row>
-    <row r="56" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>35</v>
-      </c>
-      <c r="B56">
-        <v>2844</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>37</v>
-      </c>
-      <c r="B57">
-        <v>2790</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="60" spans="1:8" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="61" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D61" s="6"/>
-    </row>
-    <row r="62" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>40</v>
-      </c>
-      <c r="B62" t="s">
-        <v>1</v>
-      </c>
-      <c r="D62" s="6"/>
-    </row>
-    <row r="63" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>41</v>
-      </c>
-      <c r="B63">
-        <v>1</v>
-      </c>
-      <c r="D63" s="6"/>
-    </row>
-    <row r="64" spans="1:8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B64" s="7">
-        <v>3034</v>
-      </c>
-      <c r="D64" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>